<commit_message>
Record the screenshot-testing round in the QA sheet
Eleven new stories (US-31..US-41) covering the areas the existing suite did
not: phone layout density, chart plot-area use and aspect ratio, table
legibility at 375px, the drill-in panel, footnote flow, dead controls in
empty states, sticky scrolling, and breakpoint changes.

Six of the eleven failed on first test and are fixed. All were found by
looking at rendered pages — the geometry checks that preceded them reported
every one of these views as correct, because the elements were present and
correctly sized in each case.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/user_stories.xlsx
+++ b/qa/user_stories.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,9 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
@@ -82,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -98,6 +101,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1830,6 +1837,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="E33" s="5" t="inlineStr">
         <is>
@@ -1848,6 +1856,530 @@
       </c>
       <c r="F34" s="6" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>US-31</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Mobile layout</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>As a phone user, I reach real data without a long scroll</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Load / at 375x812, measure first board row</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Board content reachable in the first screen or just below</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>First row at y=1063 on an 812px screen: controls block 236px tall, board explanation 10 lines, search and toggle each a full row</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>Scoring+Defense share a row, explanations clamp to 3 lines behind 'What this shows', search+toggle share a row; first row y=833</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>US-32</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>As a reader, the weekly chart uses its plot area</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Screenshot trend chart at 375 and 1280</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Series fill the plot; differences legible</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>y-axis hard-floored at 0.8 while the highest weekly score in 13 seasons is 0.574, so a quarter of the plot was always empty</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>Ceiling 0.6 — still fixed so seasons stay comparable, still pinned at 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>US-33</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>As a phone user, the scatter keeps a readable aspect ratio</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Screenshot calibration scatter at 375</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Near-square so the diagonal is meaningful</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>351x333 (1.05:1); axis labels and quadrant notes legible; dots r=4</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>US-34</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Tables</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>As a reader, the cross-season table is legible on a phone</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Screenshot career table at 375</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>One line per source; interval plot readable</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Monogram chip and full name rendered side by side in a 124px wrapped cell: 54px rows and the interval plot squeezed to 62px</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>Chip hidden on narrow; rows 34px, plot 86px</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>US-35</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Tables</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>As a reader, the interval plot's zero line is unmistakable</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Inspect .fp at 375 and 1280</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Zero rule clearly visible — an interval touching it is the finding</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>1px hairline in --baseline, the faintest token; lost against the row</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Uses --muted and overhangs the row</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>US-36</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Drill-in</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>As a drafter, the player history panel shows which season each row is</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Click a board row at 375</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Season column present against every row</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Season column hidden: the mobile rule hiding the board's rank number was unscoped and also matched rows of the nested history table</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>Rule scoped to the board's own thead/tbody rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>US-37</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>As a reader, footnotes read as sentences</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Screenshot leaderboard footnote at 375</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Inline link flows within the sentence</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>'Across all seasons' collapsed into a 3-line column mid-sentence: .chart-note was display:flex so the anchor became a flex item at min-content width</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>display:block</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>US-38</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Empty states</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>As a reader, controls that do nothing are not shown</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Load a format with no board; IDP lens; no-match search</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>No dead controls</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Source-column toggle rendered as a blank 351x40 button — every early return in renderBoard skipped the code that labels it</t>
+        </is>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>setSrcToggle() on every path; hidden unless a table was drawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>US-39</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Scrolling</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>As a drafter, the board header and player column stay pinned</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Scroll board vertically and horizontally at 375</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>thead and .pcol remain visible</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Sticky verified visually under internal scroll and by geometry at max scrollLeft</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>US-40</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Scrolling</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>As a phone user, no section scrolls the page sideways</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Measure every scroll container at 375, 3 seasons x 3 formats</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Page never overflows; wide tables scroll inside their own box</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Only the 13-season matrix scrolls internally, with a sticky source column</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>US-41</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Responsive</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>As a user rotating my phone, the layout follows</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Cross the 640 and 820 breakpoints</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Columns, headings and charts re-resolve</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Board columns re-resolve against the live viewport; explicit toggle still wins; charts redraw on resize, orientationchange and a staged post-layout check</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Pass on first test</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Failed and fixed</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Total stories</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>All retests passing</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>